<commit_message>
update sesi 1 september
</commit_message>
<xml_diff>
--- a/test/list/panjalu/sandingtaman/list_sandingtaman_2.xlsx
+++ b/test/list/panjalu/sandingtaman/list_sandingtaman_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\wdio-dds\test\list\panjalu\sandingtaman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A37A6B-34E1-4A46-BED9-D7023E667BA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE99B50-F830-4573-8974-E5BEDD97E3C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4A4170CD-5F29-480B-944E-1B0FEA867C5C}"/>
   </bookViews>
@@ -16,6 +16,9 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="conf" sheetId="2" r:id="rId2"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId3"/>
+  </externalReferences>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -26,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="156">
   <si>
     <t>nama</t>
   </si>
@@ -254,6 +257,246 @@
   </si>
   <si>
     <t>2023-08-23</t>
+  </si>
+  <si>
+    <t>2023-08-05</t>
+  </si>
+  <si>
+    <t>DENI ANSORI</t>
+  </si>
+  <si>
+    <t>Jalan tidak ramah lingkungan, tanpa pohon atau taman penyerap polusi.</t>
+  </si>
+  <si>
+    <t>2023-08-07</t>
+  </si>
+  <si>
+    <t>SAPRI</t>
+  </si>
+  <si>
+    <t>Marka jalan yang pudar atau tidak terlihat jelas, meningkatkan risiko kecelakaan.</t>
+  </si>
+  <si>
+    <t>ADAH</t>
+  </si>
+  <si>
+    <t>Kurangnya jalan alternatif untuk mengurangi kepadatan lalu lintas di ruas jalan utama.</t>
+  </si>
+  <si>
+    <t>MUHAMMAD FARIZ</t>
+  </si>
+  <si>
+    <t>Tidak adanya jalur pejalan kaki yang terpisah, menyebabkan konflik dengan kendaraan.</t>
+  </si>
+  <si>
+    <t>ABDULOH</t>
+  </si>
+  <si>
+    <t>Kurangnya pengawasan terhadap keselamatan jalan, memicu pelanggaran lalu lintas.</t>
+  </si>
+  <si>
+    <t>MAEMANAH</t>
+  </si>
+  <si>
+    <t>Kurangnya perencanaan jalan yang memadai, mengakibatkan kepadatan lalu lintas dan ketidaknyamanan pengguna jalan.</t>
+  </si>
+  <si>
+    <t>2023-08-08</t>
+  </si>
+  <si>
+    <t>MUHAMAD MIFTAHUL ULLUM</t>
+  </si>
+  <si>
+    <t>Lampu jalan di depan rumah saya tidak menyala ketika malam.</t>
+  </si>
+  <si>
+    <t>MUHAMAD ALFAN NAZMUDIN</t>
+  </si>
+  <si>
+    <t>Jalan di sekitar lingkungan kami berlubang dan perlu diperbaiki.</t>
+  </si>
+  <si>
+    <t>MUSA</t>
+  </si>
+  <si>
+    <t>Sampah di taman umum tidak dibersihkan secara teratur.</t>
+  </si>
+  <si>
+    <t>RUKANAH</t>
+  </si>
+  <si>
+    <t>Sistem drainase di daerah kami tidak berfungsi dengan baik saat hujan.</t>
+  </si>
+  <si>
+    <t>ARIPIN</t>
+  </si>
+  <si>
+    <t>Ada kebisingan berlebihan dari pabrik yang mengganggu kenyamanan tinggal kami.</t>
+  </si>
+  <si>
+    <t>2023-08-09</t>
+  </si>
+  <si>
+    <t>MAMAH</t>
+  </si>
+  <si>
+    <t>Fasilitas olahraga seperti lapangan sepak bola dan lapangan basket rusak dan tidak diperbaiki.</t>
+  </si>
+  <si>
+    <t>AI AFIFAH NURFADILAH</t>
+  </si>
+  <si>
+    <t>Tidak ada tempat penampungan sampah yang cukup di sekitar kami.</t>
+  </si>
+  <si>
+    <t>RISMA NURHADAYANTI</t>
+  </si>
+  <si>
+    <t>Air minum dari kran di rumah kami terasa kotor dan berbau.</t>
+  </si>
+  <si>
+    <t>ALIFAH ALFA KAMALA</t>
+  </si>
+  <si>
+    <t>Sekolah setempat kurang memadai dalam menyediakan fasilitas pendidikan yang memadai.</t>
+  </si>
+  <si>
+    <t>MALIHAH</t>
+  </si>
+  <si>
+    <t>Gang-gang di lingkungan kami tidak terawat dan menjadi sarang nyamuk.</t>
+  </si>
+  <si>
+    <t>2023-08-10</t>
+  </si>
+  <si>
+    <t>MUIN</t>
+  </si>
+  <si>
+    <t>Perluasan jalan di sekitar kami menyebabkan kemacetan lalu lintas yang parah.</t>
+  </si>
+  <si>
+    <t>DAYIMAH</t>
+  </si>
+  <si>
+    <t>Kualitas udara di lingkungan kami buruk karena polusi kendaraan.</t>
+  </si>
+  <si>
+    <t>HAERUDIN</t>
+  </si>
+  <si>
+    <t>Rute angkutan umum ke daerah kami tidak memadai untuk masyarakat.</t>
+  </si>
+  <si>
+    <t>IHAT SOLIHAT</t>
+  </si>
+  <si>
+    <t>Listrik sering mati dan pemadaman berlangsung lama di lingkungan kami.</t>
+  </si>
+  <si>
+    <t>JUJUN JUNAEDI</t>
+  </si>
+  <si>
+    <t>Tidak ada fasilitas kesehatan yang memadai di dekat tempat tinggal kami.</t>
+  </si>
+  <si>
+    <t>2023-08-11</t>
+  </si>
+  <si>
+    <t>IING AMIRULLAH</t>
+  </si>
+  <si>
+    <t>Tingkat kejahatan di lingkungan kami meningkat dan perlu keamanan yang lebih baik.</t>
+  </si>
+  <si>
+    <t>LINA AGUSTINA</t>
+  </si>
+  <si>
+    <t>Tidak ada tempat bermain untuk anak-anak di sekitar kami.</t>
+  </si>
+  <si>
+    <t>NAIRA ALESHA AMIRULLAH</t>
+  </si>
+  <si>
+    <t>Kualitas air di sungai atau danau terdekat tercemar dan perlu diperbaiki.</t>
+  </si>
+  <si>
+    <t>JAELANI NURSIDIK</t>
+  </si>
+  <si>
+    <t>Ruang publik seperti taman dan area hijau tidak dirawat dengan baik.</t>
+  </si>
+  <si>
+    <t>NIA KORINA</t>
+  </si>
+  <si>
+    <t>Kualitas penerangan di jalan-jalan kami buruk dan perlu ditingkatkan.</t>
+  </si>
+  <si>
+    <t>2023-08-12</t>
+  </si>
+  <si>
+    <t>ZAIDAN MUHAMMAD ARKANA</t>
+  </si>
+  <si>
+    <t>Kurangnya tempat parkir yang memadai di sekitar toko dan pusat perbelanjaan.</t>
+  </si>
+  <si>
+    <t>DENI</t>
+  </si>
+  <si>
+    <t>Kurangnya lapangan kerja di lingkungan kami membuat ekonomi warga sulit.</t>
+  </si>
+  <si>
+    <t>CUCU CAHYATI</t>
+  </si>
+  <si>
+    <t>Internet di daerah kami tidak stabil dan sering putus.</t>
+  </si>
+  <si>
+    <t>DAFA IBNU HAFIDZ</t>
+  </si>
+  <si>
+    <t>Tidak adanya aksesibilitas bagi orang dengan kebutuhan khusus di tempat umum.</t>
+  </si>
+  <si>
+    <t>YOYO CAHYO</t>
+  </si>
+  <si>
+    <t>Binatang liar seperti anjing liar menjadi masalah di lingkungan kami.</t>
+  </si>
+  <si>
+    <t>2023-08-14</t>
+  </si>
+  <si>
+    <t>MAYA KOMALASARI</t>
+  </si>
+  <si>
+    <t>Tidak ada jalur pejalan kaki yang aman di sekitar jalan-jalan utama.</t>
+  </si>
+  <si>
+    <t>SUMYATI</t>
+  </si>
+  <si>
+    <t>Tidak adanya ruang terbuka hijau yang cukup di dekat tempat tinggal kami.</t>
+  </si>
+  <si>
+    <t>MAMAN</t>
+  </si>
+  <si>
+    <t>Tidak ada layanan angkutan umum pada larut malam di wilayah kami.</t>
+  </si>
+  <si>
+    <t>KOMARUDIN</t>
+  </si>
+  <si>
+    <t>Bangunan yang ditinggalkan dan tidak terawat di sekitar kami menjadi tempat tinggal bagi tikus dan serangga.</t>
+  </si>
+  <si>
+    <t>SITI JUBAEDAH</t>
+  </si>
+  <si>
+    <t>Kurangnya tempat ibadah yang memadai di daerah kami.</t>
   </si>
 </sst>
 </file>
@@ -312,11 +555,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -344,6 +590,169 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Sheet1"/>
+      <sheetName val="conf"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1">
+        <row r="2">
+          <cell r="A2" t="str">
+            <v>Sandingtaman</v>
+          </cell>
+          <cell r="B2" t="str">
+            <v>Karoya</v>
+          </cell>
+          <cell r="C2" t="str">
+            <v>001</v>
+          </cell>
+          <cell r="D2" t="str">
+            <v>001</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="B3" t="str">
+            <v>Cipicung</v>
+          </cell>
+          <cell r="C3" t="str">
+            <v>002</v>
+          </cell>
+          <cell r="D3" t="str">
+            <v>002</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="B4" t="str">
+            <v>Nanggela</v>
+          </cell>
+          <cell r="C4" t="str">
+            <v>003</v>
+          </cell>
+          <cell r="D4" t="str">
+            <v>003</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="B5" t="str">
+            <v>Sanding</v>
+          </cell>
+          <cell r="C5" t="str">
+            <v>004</v>
+          </cell>
+          <cell r="D5" t="str">
+            <v>004</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="B6" t="str">
+            <v>Citaman</v>
+          </cell>
+          <cell r="C6" t="str">
+            <v>005</v>
+          </cell>
+          <cell r="D6" t="str">
+            <v>005</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="B7" t="str">
+            <v>Sindangjaya</v>
+          </cell>
+          <cell r="C7" t="str">
+            <v>006</v>
+          </cell>
+          <cell r="D7" t="str">
+            <v>006</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="B8" t="str">
+            <v>Cidarma</v>
+          </cell>
+          <cell r="C8" t="str">
+            <v>007</v>
+          </cell>
+          <cell r="D8" t="str">
+            <v>007</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="C9" t="str">
+            <v>008</v>
+          </cell>
+          <cell r="D9" t="str">
+            <v>008</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="C10" t="str">
+            <v>009</v>
+          </cell>
+          <cell r="D10" t="str">
+            <v>009</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="C11" t="str">
+            <v>010</v>
+          </cell>
+          <cell r="D11" t="str">
+            <v>010</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="C12" t="str">
+            <v>011</v>
+          </cell>
+          <cell r="D12" t="str">
+            <v>011</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="C13" t="str">
+            <v>012</v>
+          </cell>
+          <cell r="D13" t="str">
+            <v>012</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="C14" t="str">
+            <v>013</v>
+          </cell>
+          <cell r="D14" t="str">
+            <v>013</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="C15" t="str">
+            <v>014</v>
+          </cell>
+          <cell r="D15" t="str">
+            <v>014</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="C16" t="str">
+            <v>015</v>
+          </cell>
+          <cell r="D16" t="str">
+            <v>015</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -643,7 +1052,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{330EDF8F-AF7E-4CFD-AD2A-76F45302569C}">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14.36328125" style="1" customWidth="1"/>
@@ -691,15 +1100,15 @@
       </c>
       <c r="D2" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Cidarma</v>
+        <v>Sindangjaya</v>
       </c>
       <c r="E2" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>008</v>
+        <v>001</v>
       </c>
       <c r="F2" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>004</v>
+        <v>006</v>
       </c>
       <c r="G2" s="3" t="str">
         <f>conf!$A$2</f>
@@ -725,7 +1134,7 @@
       </c>
       <c r="D3" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Sanding</v>
+        <v>Sindangjaya</v>
       </c>
       <c r="E3" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
@@ -733,7 +1142,7 @@
       </c>
       <c r="F3" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>014</v>
+        <v>008</v>
       </c>
       <c r="G3" s="3" t="str">
         <f>conf!$A$2</f>
@@ -759,15 +1168,15 @@
       </c>
       <c r="D4" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Nanggela</v>
+        <v>Sindangjaya</v>
       </c>
       <c r="E4" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>003</v>
+        <v>009</v>
       </c>
       <c r="F4" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>006</v>
+        <v>001</v>
       </c>
       <c r="G4" s="3" t="str">
         <f>conf!$A$2</f>
@@ -793,15 +1202,15 @@
       </c>
       <c r="D5" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Citaman</v>
+        <v>Sanding</v>
       </c>
       <c r="E5" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>010</v>
+        <v>003</v>
       </c>
       <c r="F5" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>009</v>
+        <v>006</v>
       </c>
       <c r="G5" s="3" t="str">
         <f>conf!$A$2</f>
@@ -827,15 +1236,15 @@
       </c>
       <c r="D6" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Cidarma</v>
+        <v>Nanggela</v>
       </c>
       <c r="E6" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>001</v>
+        <v>003</v>
       </c>
       <c r="F6" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>003</v>
+        <v>012</v>
       </c>
       <c r="G6" s="3" t="str">
         <f>conf!$A$2</f>
@@ -865,11 +1274,11 @@
       </c>
       <c r="E7" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>003</v>
+        <v>012</v>
       </c>
       <c r="F7" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>001</v>
+        <v>015</v>
       </c>
       <c r="G7" s="3" t="str">
         <f>conf!$A$2</f>
@@ -895,15 +1304,15 @@
       </c>
       <c r="D8" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Cipicung</v>
+        <v>Citaman</v>
       </c>
       <c r="E8" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>011</v>
+        <v>001</v>
       </c>
       <c r="F8" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>011</v>
+        <v>001</v>
       </c>
       <c r="G8" s="3" t="str">
         <f>conf!$A$2</f>
@@ -929,15 +1338,15 @@
       </c>
       <c r="D9" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Citaman</v>
+        <v>Sindangjaya</v>
       </c>
       <c r="E9" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>010</v>
+        <v>002</v>
       </c>
       <c r="F9" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>006</v>
+        <v>010</v>
       </c>
       <c r="G9" s="3" t="str">
         <f>conf!$A$2</f>
@@ -963,15 +1372,15 @@
       </c>
       <c r="D10" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Nanggela</v>
+        <v>Cipicung</v>
       </c>
       <c r="E10" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>006</v>
+        <v>001</v>
       </c>
       <c r="F10" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>001</v>
+        <v>002</v>
       </c>
       <c r="G10" s="3" t="str">
         <f>conf!$A$2</f>
@@ -997,15 +1406,15 @@
       </c>
       <c r="D11" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Citaman</v>
+        <v>Nanggela</v>
       </c>
       <c r="E11" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>008</v>
+        <v>013</v>
       </c>
       <c r="F11" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>006</v>
+        <v>008</v>
       </c>
       <c r="G11" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1031,15 +1440,15 @@
       </c>
       <c r="D12" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Nanggela</v>
+        <v>Sanding</v>
       </c>
       <c r="E12" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>015</v>
+        <v>002</v>
       </c>
       <c r="F12" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>011</v>
+        <v>014</v>
       </c>
       <c r="G12" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1065,15 +1474,15 @@
       </c>
       <c r="D13" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Cidarma</v>
+        <v>Cipicung</v>
       </c>
       <c r="E13" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>014</v>
+        <v>010</v>
       </c>
       <c r="F13" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>013</v>
+        <v>006</v>
       </c>
       <c r="G13" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1099,15 +1508,15 @@
       </c>
       <c r="D14" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Citaman</v>
+        <v>Cipicung</v>
       </c>
       <c r="E14" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>015</v>
+        <v>006</v>
       </c>
       <c r="F14" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>003</v>
+        <v>006</v>
       </c>
       <c r="G14" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1133,15 +1542,15 @@
       </c>
       <c r="D15" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Sanding</v>
+        <v>Citaman</v>
       </c>
       <c r="E15" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>013</v>
+        <v>010</v>
       </c>
       <c r="F15" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>011</v>
+        <v>003</v>
       </c>
       <c r="G15" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1167,15 +1576,15 @@
       </c>
       <c r="D16" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Cipicung</v>
+        <v>Nanggela</v>
       </c>
       <c r="E16" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>013</v>
+        <v>001</v>
       </c>
       <c r="F16" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>002</v>
+        <v>013</v>
       </c>
       <c r="G16" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1201,15 +1610,15 @@
       </c>
       <c r="D17" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Nanggela</v>
+        <v>Karoya</v>
       </c>
       <c r="E17" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>005</v>
+        <v>012</v>
       </c>
       <c r="F17" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>002</v>
+        <v>010</v>
       </c>
       <c r="G17" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1235,15 +1644,15 @@
       </c>
       <c r="D18" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Cidarma</v>
+        <v>Karoya</v>
       </c>
       <c r="E18" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>002</v>
+        <v>012</v>
       </c>
       <c r="F18" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>005</v>
+        <v>003</v>
       </c>
       <c r="G18" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1269,15 +1678,15 @@
       </c>
       <c r="D19" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Cipicung</v>
+        <v>Sindangjaya</v>
       </c>
       <c r="E19" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>009</v>
+        <v>014</v>
       </c>
       <c r="F19" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>009</v>
+        <v>013</v>
       </c>
       <c r="G19" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1303,15 +1712,15 @@
       </c>
       <c r="D20" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Citaman</v>
+        <v>Karoya</v>
       </c>
       <c r="E20" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>015</v>
+        <v>002</v>
       </c>
       <c r="F20" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>010</v>
+        <v>011</v>
       </c>
       <c r="G20" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1337,15 +1746,15 @@
       </c>
       <c r="D21" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Nanggela</v>
+        <v>Citaman</v>
       </c>
       <c r="E21" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>005</v>
+        <v>002</v>
       </c>
       <c r="F21" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>001</v>
+        <v>004</v>
       </c>
       <c r="G21" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1371,15 +1780,15 @@
       </c>
       <c r="D22" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
-        <v>Nanggela</v>
+        <v>Karoya</v>
       </c>
       <c r="E22" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
-        <v>007</v>
+        <v>005</v>
       </c>
       <c r="F22" s="2" t="str">
         <f ca="1">INDEX(conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
-        <v>012</v>
+        <v>015</v>
       </c>
       <c r="G22" s="3" t="str">
         <f>conf!$A$2</f>
@@ -1394,60 +1803,1084 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="3"/>
+      <c r="A23">
+        <v>25</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D23" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sindangjaya</v>
+      </c>
+      <c r="E23" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>014</v>
+      </c>
+      <c r="F23" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>003</v>
+      </c>
+      <c r="G23" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H23" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="3"/>
+      <c r="A24">
+        <v>26</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D24" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Nanggela</v>
+      </c>
+      <c r="E24" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>013</v>
+      </c>
+      <c r="F24" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>013</v>
+      </c>
+      <c r="G24" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H24" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="3"/>
+      <c r="A25">
+        <v>27</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D25" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Karoya</v>
+      </c>
+      <c r="E25" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>003</v>
+      </c>
+      <c r="F25" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>003</v>
+      </c>
+      <c r="G25" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H25" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="3"/>
+      <c r="A26">
+        <v>28</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sanding</v>
+      </c>
+      <c r="E26" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>010</v>
+      </c>
+      <c r="F26" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>002</v>
+      </c>
+      <c r="G26" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H26" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="3"/>
+      <c r="A27">
+        <v>29</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D27" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Nanggela</v>
+      </c>
+      <c r="E27" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>013</v>
+      </c>
+      <c r="F27" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>009</v>
+      </c>
+      <c r="G27" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H27" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="3"/>
+      <c r="A28">
+        <v>30</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D28" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Karoya</v>
+      </c>
+      <c r="E28" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>010</v>
+      </c>
+      <c r="F28" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>003</v>
+      </c>
+      <c r="G28" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H28" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="3"/>
+      <c r="A29">
+        <v>31</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D29" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sindangjaya</v>
+      </c>
+      <c r="E29" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>012</v>
+      </c>
+      <c r="F29" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>003</v>
+      </c>
+      <c r="G29" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H29" t="s">
+        <v>92</v>
+      </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="3"/>
+      <c r="A30">
+        <v>32</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D30" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Cidarma</v>
+      </c>
+      <c r="E30" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>004</v>
+      </c>
+      <c r="F30" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>012</v>
+      </c>
+      <c r="G30" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H30" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>33</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D31" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Cidarma</v>
+      </c>
+      <c r="E31" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>003</v>
+      </c>
+      <c r="F31" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>010</v>
+      </c>
+      <c r="G31" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>34</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D32" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Cipicung</v>
+      </c>
+      <c r="E32" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>003</v>
+      </c>
+      <c r="F32" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>006</v>
+      </c>
+      <c r="G32" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>35</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D33" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sanding</v>
+      </c>
+      <c r="E33" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>013</v>
+      </c>
+      <c r="F33" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>009</v>
+      </c>
+      <c r="G33" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>36</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D34" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Karoya</v>
+      </c>
+      <c r="E34" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>002</v>
+      </c>
+      <c r="F34" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>013</v>
+      </c>
+      <c r="G34" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>37</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D35" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sindangjaya</v>
+      </c>
+      <c r="E35" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>005</v>
+      </c>
+      <c r="F35" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>013</v>
+      </c>
+      <c r="G35" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>38</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D36" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Karoya</v>
+      </c>
+      <c r="E36" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>001</v>
+      </c>
+      <c r="F36" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>002</v>
+      </c>
+      <c r="G36" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>39</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D37" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Nanggela</v>
+      </c>
+      <c r="E37" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>010</v>
+      </c>
+      <c r="F37" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>003</v>
+      </c>
+      <c r="G37" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>40</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D38" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Karoya</v>
+      </c>
+      <c r="E38" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>004</v>
+      </c>
+      <c r="F38" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>001</v>
+      </c>
+      <c r="G38" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>41</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D39" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sanding</v>
+      </c>
+      <c r="E39" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>004</v>
+      </c>
+      <c r="F39" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>015</v>
+      </c>
+      <c r="G39" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H39" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>42</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D40" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Nanggela</v>
+      </c>
+      <c r="E40" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>013</v>
+      </c>
+      <c r="F40" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>006</v>
+      </c>
+      <c r="G40" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>43</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D41" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sindangjaya</v>
+      </c>
+      <c r="E41" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>006</v>
+      </c>
+      <c r="F41" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>011</v>
+      </c>
+      <c r="G41" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>44</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D42" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Cidarma</v>
+      </c>
+      <c r="E42" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>002</v>
+      </c>
+      <c r="F42" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>012</v>
+      </c>
+      <c r="G42" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>45</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D43" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Cidarma</v>
+      </c>
+      <c r="E43" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>012</v>
+      </c>
+      <c r="F43" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>011</v>
+      </c>
+      <c r="G43" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>46</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D44" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sanding</v>
+      </c>
+      <c r="E44" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>013</v>
+      </c>
+      <c r="F44" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>004</v>
+      </c>
+      <c r="G44" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>47</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D45" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sanding</v>
+      </c>
+      <c r="E45" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>015</v>
+      </c>
+      <c r="F45" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>014</v>
+      </c>
+      <c r="G45" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>48</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D46" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Citaman</v>
+      </c>
+      <c r="E46" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>015</v>
+      </c>
+      <c r="F46" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>001</v>
+      </c>
+      <c r="G46" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>49</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D47" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Cidarma</v>
+      </c>
+      <c r="E47" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>015</v>
+      </c>
+      <c r="F47" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>011</v>
+      </c>
+      <c r="G47" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>50</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D48" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sanding</v>
+      </c>
+      <c r="E48" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>009</v>
+      </c>
+      <c r="F48" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>013</v>
+      </c>
+      <c r="G48" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H48" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>51</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D49" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Nanggela</v>
+      </c>
+      <c r="E49" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>004</v>
+      </c>
+      <c r="F49" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>008</v>
+      </c>
+      <c r="G49" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>52</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D50" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Cidarma</v>
+      </c>
+      <c r="E50" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>008</v>
+      </c>
+      <c r="F50" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>014</v>
+      </c>
+      <c r="G50" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H50" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>53</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D51" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sanding</v>
+      </c>
+      <c r="E51" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>002</v>
+      </c>
+      <c r="F51" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>012</v>
+      </c>
+      <c r="G51" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H51" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>54</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D52" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Cidarma</v>
+      </c>
+      <c r="E52" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>005</v>
+      </c>
+      <c r="F52" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>001</v>
+      </c>
+      <c r="G52" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H52" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A53">
+        <v>55</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D53" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Citaman</v>
+      </c>
+      <c r="E53" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>005</v>
+      </c>
+      <c r="F53" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>009</v>
+      </c>
+      <c r="G53" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H53" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A54">
+        <v>56</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D54" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Citaman</v>
+      </c>
+      <c r="E54" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>001</v>
+      </c>
+      <c r="F54" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>004</v>
+      </c>
+      <c r="G54" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H54" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A55">
+        <v>57</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D55" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sanding</v>
+      </c>
+      <c r="E55" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>006</v>
+      </c>
+      <c r="F55" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>013</v>
+      </c>
+      <c r="G55" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H55" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A56">
+        <v>58</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D56" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Karoya</v>
+      </c>
+      <c r="E56" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>004</v>
+      </c>
+      <c r="F56" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>002</v>
+      </c>
+      <c r="G56" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H56" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A57">
+        <v>59</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D57" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Nanggela</v>
+      </c>
+      <c r="E57" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>008</v>
+      </c>
+      <c r="F57" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>010</v>
+      </c>
+      <c r="G57" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H57" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A58">
+        <v>60</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="D58" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,7),1)</f>
+        <v>Sindangjaya</v>
+      </c>
+      <c r="E58" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),3)</f>
+        <v>012</v>
+      </c>
+      <c r="F58" s="2" t="str">
+        <f ca="1">INDEX([1]conf!$B$2:$D$16,RANDBETWEEN(1,15),2)</f>
+        <v>002</v>
+      </c>
+      <c r="G58" s="3" t="str">
+        <f>[1]conf!$A$2</f>
+        <v>Sandingtaman</v>
+      </c>
+      <c r="H58" t="s">
+        <v>155</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>